<commit_message>
Trinsic - Most Conversations and Some Trades Tested.
</commit_message>
<xml_diff>
--- a/spoilers/trades.xlsx
+++ b/spoilers/trades.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2B2162F-053E-4181-9F0E-85BB8D388381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27146181-CC5C-4EE1-AA02-8B4CDBF28613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="196">
   <si>
     <t>NBT Villager Trade Template</t>
   </si>
@@ -605,12 +605,77 @@
   <si>
     <t>rotten_flesh</t>
   </si>
+  <si>
+    <t>Trinsic</t>
+  </si>
+  <si>
+    <t>Swindrik</t>
+  </si>
+  <si>
+    <t>Wizard</t>
+  </si>
+  <si>
+    <t>paper</t>
+  </si>
+  <si>
+    <t>Gating Trade L1 to L2; "a worthy exchange!"</t>
+  </si>
+  <si>
+    <t>chorus_fruit</t>
+  </si>
+  <si>
+    <t>title: TELEPORT POTIONS
+author: Swindrik
+[PAGE]
+About POTIONS:
+Every VIRTUE has always had a MOONGATE and for each a TOWN was built nearby. 
+We use the power of the moongates and chorus fruit to TELEPORT between towns.
+In general, it needs a container, a carrier, a symbolic, and an edible.
+[PAGE]
+Potion List:
+B1. Return Potion    - GB, RD, D, ...and a seed.
+B5. Potion of Honor  - WB, CF, C, ...and a fungus.
+B6. Ptn/Compassion   - GB, RD, BR, and BM 
+[PAGE]
+The RETURN POTION is made from the simplest ingredients -- dirt, wheat seeds, and 1 redstone dust, mixed into a glass bottle.
+The trick, really, is to find a good source of redstone dust... And, some CLERICS are said to hold GREAT amounts of it!</t>
+  </si>
+  <si>
+    <t>Zajac</t>
+  </si>
+  <si>
+    <t>redstone_dust</t>
+  </si>
+  <si>
+    <t>Gating trade L1 to L2; "here's your change. Enjoy your stay".  (He opens iron door to room. It shuts when plate inside is stepped upon)</t>
+  </si>
+  <si>
+    <t>No further leveling required. He says "here's your change. Enjoy your stay".  (He opens iron door to room. It shuts when plate inside is stepped upon)</t>
+  </si>
+  <si>
+    <t>Terran</t>
+  </si>
+  <si>
+    <t>Bartender</t>
+  </si>
+  <si>
+    <t>carrot</t>
+  </si>
+  <si>
+    <t>milk_bucket</t>
+  </si>
+  <si>
+    <t>sugar</t>
+  </si>
+  <si>
+    <t>cooked_rabbit</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -658,8 +723,21 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -681,6 +759,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -738,7 +822,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -888,6 +972,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1317,7 +1410,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L317"/>
+  <dimension ref="A1:L1048576"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1328,7 +1421,7 @@
     <col min="6" max="6" width="10" style="27" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
     <col min="8" max="8" width="10" style="27" customWidth="1"/>
-    <col min="9" max="9" width="40" style="44" customWidth="1"/>
+    <col min="9" max="9" width="75.88671875" style="44" customWidth="1"/>
     <col min="10" max="10" width="10" style="53" customWidth="1"/>
     <col min="11" max="11" width="11.44140625" style="53" customWidth="1"/>
     <col min="12" max="12" width="34" style="52" customWidth="1"/>
@@ -4264,144 +4357,356 @@
       </c>
       <c r="L83" s="48"/>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A84" s="5"/>
-      <c r="B84" s="5"/>
-      <c r="C84" s="5"/>
-      <c r="D84" s="26"/>
-      <c r="E84" s="5"/>
-      <c r="F84" s="26"/>
-      <c r="G84" s="5"/>
-      <c r="H84" s="26"/>
+    <row r="84" spans="1:12" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A84" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="B84" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C84" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D84" s="26">
+        <v>1</v>
+      </c>
+      <c r="E84" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="F84" s="26">
+        <v>1</v>
+      </c>
+      <c r="G84" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="H84" s="26">
+        <v>2</v>
+      </c>
       <c r="I84" s="41"/>
-      <c r="J84" s="28"/>
-      <c r="K84" s="28"/>
-      <c r="L84" s="48"/>
+      <c r="J84" s="28">
+        <v>999999</v>
+      </c>
+      <c r="K84" s="28">
+        <v>5</v>
+      </c>
+      <c r="L84" s="59" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A85" s="5"/>
-      <c r="B85" s="5"/>
-      <c r="C85" s="5"/>
-      <c r="D85" s="26"/>
-      <c r="E85" s="5"/>
-      <c r="F85" s="26"/>
-      <c r="G85" s="5"/>
-      <c r="H85" s="26"/>
-      <c r="I85" s="41"/>
-      <c r="J85" s="28"/>
-      <c r="K85" s="28"/>
-      <c r="L85" s="48"/>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A86" s="5"/>
-      <c r="B86" s="5"/>
-      <c r="C86" s="5"/>
-      <c r="D86" s="26"/>
-      <c r="E86" s="5"/>
-      <c r="F86" s="26"/>
-      <c r="G86" s="5"/>
-      <c r="H86" s="26"/>
-      <c r="I86" s="41"/>
-      <c r="J86" s="28"/>
-      <c r="K86" s="28"/>
-      <c r="L86" s="48"/>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A87" s="5"/>
-      <c r="B87" s="5"/>
-      <c r="C87" s="5"/>
-      <c r="D87" s="26"/>
-      <c r="E87" s="5"/>
-      <c r="F87" s="26"/>
-      <c r="G87" s="5"/>
-      <c r="H87" s="26"/>
-      <c r="I87" s="41"/>
-      <c r="J87" s="28"/>
-      <c r="K87" s="28"/>
-      <c r="L87" s="48"/>
-    </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A88" s="5"/>
-      <c r="B88" s="5"/>
-      <c r="C88" s="5"/>
-      <c r="D88" s="26"/>
-      <c r="E88" s="5"/>
-      <c r="F88" s="26"/>
-      <c r="G88" s="5"/>
-      <c r="H88" s="26"/>
+      <c r="A85" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C85" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D85" s="26">
+        <v>2</v>
+      </c>
+      <c r="E85" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F85" s="26">
+        <v>3</v>
+      </c>
+      <c r="G85" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="H85" s="26">
+        <v>2</v>
+      </c>
+      <c r="I85" s="43"/>
+      <c r="J85" s="28">
+        <v>999999</v>
+      </c>
+      <c r="K85" s="29">
+        <v>30</v>
+      </c>
+      <c r="L85" s="59"/>
+    </row>
+    <row r="86" spans="1:12" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A86" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="B86" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C86" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D86" s="26">
+        <v>2</v>
+      </c>
+      <c r="E86" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="F86" s="26">
+        <v>1</v>
+      </c>
+      <c r="G86" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="H86" s="26">
+        <v>1</v>
+      </c>
+      <c r="I86" s="43"/>
+      <c r="J86" s="28">
+        <v>999999</v>
+      </c>
+      <c r="K86" s="29">
+        <v>30</v>
+      </c>
+      <c r="L86" s="59" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" s="27" customFormat="1" ht="276" x14ac:dyDescent="0.3">
+      <c r="A87" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="B87" s="28" t="s">
+        <v>180</v>
+      </c>
+      <c r="C87" s="28" t="s">
+        <v>181</v>
+      </c>
+      <c r="D87" s="28">
+        <v>3</v>
+      </c>
+      <c r="E87" s="28" t="s">
+        <v>184</v>
+      </c>
+      <c r="F87" s="28">
+        <v>1</v>
+      </c>
+      <c r="G87" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="H87" s="33">
+        <v>1</v>
+      </c>
+      <c r="I87" s="57" t="s">
+        <v>185</v>
+      </c>
+      <c r="J87" s="28">
+        <v>999999</v>
+      </c>
+      <c r="K87" s="28">
+        <v>5</v>
+      </c>
+      <c r="L87" s="59" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" ht="53.4" x14ac:dyDescent="0.3">
+      <c r="A88" s="56" t="s">
+        <v>179</v>
+      </c>
+      <c r="B88" s="58" t="s">
+        <v>186</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="D88" s="26">
+        <v>1</v>
+      </c>
+      <c r="E88" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="F88" s="26">
+        <v>2</v>
+      </c>
+      <c r="G88" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H88" s="26">
+        <v>1</v>
+      </c>
       <c r="I88" s="41"/>
-      <c r="J88" s="28"/>
-      <c r="K88" s="28"/>
-      <c r="L88" s="48"/>
-    </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A89" s="5"/>
-      <c r="B89" s="5"/>
-      <c r="C89" s="5"/>
-      <c r="D89" s="26"/>
-      <c r="E89" s="5"/>
-      <c r="F89" s="26"/>
-      <c r="G89" s="5"/>
-      <c r="H89" s="26"/>
+      <c r="J88" s="28">
+        <v>1</v>
+      </c>
+      <c r="K88" s="28">
+        <v>10</v>
+      </c>
+      <c r="L88" s="48" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" ht="53.4" x14ac:dyDescent="0.3">
+      <c r="A89" s="56" t="s">
+        <v>179</v>
+      </c>
+      <c r="B89" s="58" t="s">
+        <v>186</v>
+      </c>
+      <c r="C89" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="D89" s="26">
+        <v>2</v>
+      </c>
+      <c r="E89" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="F89" s="26">
+        <v>2</v>
+      </c>
+      <c r="G89" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H89" s="26">
+        <v>1</v>
+      </c>
       <c r="I89" s="41"/>
-      <c r="J89" s="28"/>
-      <c r="K89" s="28"/>
-      <c r="L89" s="48"/>
+      <c r="J89" s="28">
+        <v>999999</v>
+      </c>
+      <c r="K89" s="28">
+        <v>0</v>
+      </c>
+      <c r="L89" s="48" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A90" s="5"/>
-      <c r="B90" s="5"/>
-      <c r="C90" s="5"/>
-      <c r="D90" s="26"/>
-      <c r="E90" s="5"/>
-      <c r="F90" s="26"/>
-      <c r="G90" s="5"/>
-      <c r="H90" s="26"/>
+      <c r="A90" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="B90" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C90" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="D90" s="26">
+        <v>1</v>
+      </c>
+      <c r="E90" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="F90" s="26">
+        <v>1</v>
+      </c>
+      <c r="G90" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="H90" s="26">
+        <v>2</v>
+      </c>
       <c r="I90" s="41"/>
-      <c r="J90" s="28"/>
-      <c r="K90" s="28"/>
-      <c r="L90" s="48"/>
+      <c r="J90" s="28">
+        <v>999999</v>
+      </c>
+      <c r="K90" s="28">
+        <v>0</v>
+      </c>
+      <c r="L90" s="59"/>
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A91" s="5"/>
-      <c r="B91" s="5"/>
-      <c r="C91" s="5"/>
-      <c r="D91" s="26"/>
-      <c r="E91" s="5"/>
-      <c r="F91" s="26"/>
-      <c r="G91" s="5"/>
-      <c r="H91" s="26"/>
+      <c r="A91" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="B91" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C91" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="D91" s="26">
+        <v>1</v>
+      </c>
+      <c r="E91" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="F91" s="26">
+        <v>1</v>
+      </c>
+      <c r="G91" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="H91" s="26">
+        <v>1</v>
+      </c>
       <c r="I91" s="41"/>
-      <c r="J91" s="28"/>
-      <c r="K91" s="28"/>
+      <c r="J91" s="28">
+        <v>999999</v>
+      </c>
+      <c r="K91" s="28">
+        <v>0</v>
+      </c>
       <c r="L91" s="48"/>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A92" s="5"/>
-      <c r="B92" s="5"/>
-      <c r="C92" s="5"/>
-      <c r="D92" s="26"/>
-      <c r="E92" s="5"/>
-      <c r="F92" s="26"/>
-      <c r="G92" s="5"/>
-      <c r="H92" s="26"/>
+      <c r="A92" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="B92" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C92" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="D92" s="26">
+        <v>1</v>
+      </c>
+      <c r="E92" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="F92" s="26">
+        <v>1</v>
+      </c>
+      <c r="G92" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="H92" s="26">
+        <v>1</v>
+      </c>
       <c r="I92" s="41"/>
-      <c r="J92" s="28"/>
-      <c r="K92" s="28"/>
+      <c r="J92" s="28">
+        <v>999999</v>
+      </c>
+      <c r="K92" s="28">
+        <v>0</v>
+      </c>
       <c r="L92" s="48"/>
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A93" s="5"/>
-      <c r="B93" s="5"/>
-      <c r="C93" s="5"/>
-      <c r="D93" s="26"/>
-      <c r="E93" s="5"/>
-      <c r="F93" s="26"/>
-      <c r="G93" s="5"/>
-      <c r="H93" s="26"/>
+      <c r="A93" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="B93" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C93" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="D93" s="26">
+        <v>1</v>
+      </c>
+      <c r="E93" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="F93" s="26">
+        <v>2</v>
+      </c>
+      <c r="G93" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="H93" s="26">
+        <v>1</v>
+      </c>
       <c r="I93" s="41"/>
-      <c r="J93" s="28"/>
-      <c r="K93" s="28"/>
+      <c r="J93" s="28">
+        <v>999999</v>
+      </c>
+      <c r="K93" s="28">
+        <v>0</v>
+      </c>
       <c r="L93" s="48"/>
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.3">
@@ -7540,9 +7845,42 @@
       <c r="K317" s="28"/>
       <c r="L317" s="48"/>
     </row>
+    <row r="318" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A318" s="5"/>
+      <c r="B318" s="5"/>
+      <c r="C318" s="5"/>
+      <c r="D318" s="26"/>
+      <c r="E318" s="5"/>
+      <c r="F318" s="26"/>
+      <c r="G318" s="5"/>
+      <c r="H318" s="26"/>
+      <c r="I318" s="41"/>
+      <c r="J318" s="28"/>
+      <c r="K318" s="28"/>
+      <c r="L318" s="48"/>
+    </row>
+    <row r="319" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A319" s="5"/>
+      <c r="B319" s="5"/>
+      <c r="C319" s="5"/>
+      <c r="D319" s="26"/>
+      <c r="E319" s="5"/>
+      <c r="F319" s="26"/>
+      <c r="G319" s="5"/>
+      <c r="H319" s="26"/>
+      <c r="I319" s="41"/>
+      <c r="J319" s="28"/>
+      <c r="K319" s="28"/>
+      <c r="L319" s="48"/>
+    </row>
+    <row r="1048576" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1048576" s="5" t="s">
+        <v>190</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" sqref="D51:D57 D2:D43 D59:D72 D74:D317" xr:uid="{00000000-0002-0000-0100-000000000000}">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="D51:D57 D2:D43 D59:D72 D74:D319" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>